<commit_message>
Round 36 fixture: month counts rounded where the timeline reads them
The sweep moves each input by -15%, so construction (18) and hold (24)
months became 15.3 and 20.4: no period matched the sale month, the model
had no sale, and its XIRR had no unique root. The timeline now reads the
counts rounded to whole months, as a model would; base results unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016o4U1piqjugt3oSK2Yqgfb
</commit_message>
<xml_diff>
--- a/estatemaster-agent/tests/fixtures/models/r35_dev_monthly_usd.xlsx
+++ b/estatemaster-agent/tests/fixtures/models/r35_dev_monthly_usd.xlsx
@@ -558,7 +558,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -589,6 +589,10 @@
       <c r="B4" s="0" t="n">
         <v>18</v>
       </c>
+      <c r="C4" s="0" t="n">
+        <f aca="false">ROUND(B4,0)</f>
+        <v>18</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
@@ -611,6 +615,10 @@
         <v>18</v>
       </c>
       <c r="B7" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <f aca="false">ROUND(B7,0)</f>
         <v>24</v>
       </c>
     </row>
@@ -1133,179 +1141,179 @@
         <v>26</v>
       </c>
       <c r="B7" s="0" t="n">
-        <f aca="false">IF(AND(B$3&gt;=1,B$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(B$3&gt;=1,B$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="C7" s="0" t="n">
-        <f aca="false">IF(AND(C$3&gt;=1,C$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(C$3&gt;=1,C$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="D7" s="0" t="n">
-        <f aca="false">IF(AND(D$3&gt;=1,D$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(D$3&gt;=1,D$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="E7" s="0" t="n">
-        <f aca="false">IF(AND(E$3&gt;=1,E$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(E$3&gt;=1,E$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="F7" s="0" t="n">
-        <f aca="false">IF(AND(F$3&gt;=1,F$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(F$3&gt;=1,F$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="G7" s="0" t="n">
-        <f aca="false">IF(AND(G$3&gt;=1,G$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(G$3&gt;=1,G$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="H7" s="0" t="n">
-        <f aca="false">IF(AND(H$3&gt;=1,H$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(H$3&gt;=1,H$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="I7" s="0" t="n">
-        <f aca="false">IF(AND(I$3&gt;=1,I$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(I$3&gt;=1,I$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="J7" s="0" t="n">
-        <f aca="false">IF(AND(J$3&gt;=1,J$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(J$3&gt;=1,J$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="K7" s="0" t="n">
-        <f aca="false">IF(AND(K$3&gt;=1,K$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(K$3&gt;=1,K$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="L7" s="0" t="n">
-        <f aca="false">IF(AND(L$3&gt;=1,L$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(L$3&gt;=1,L$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="M7" s="0" t="n">
-        <f aca="false">IF(AND(M$3&gt;=1,M$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(M$3&gt;=1,M$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="N7" s="0" t="n">
-        <f aca="false">IF(AND(N$3&gt;=1,N$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(N$3&gt;=1,N$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="O7" s="0" t="n">
-        <f aca="false">IF(AND(O$3&gt;=1,O$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(O$3&gt;=1,O$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="P7" s="0" t="n">
-        <f aca="false">IF(AND(P$3&gt;=1,P$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(P$3&gt;=1,P$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="Q7" s="0" t="n">
-        <f aca="false">IF(AND(Q$3&gt;=1,Q$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(Q$3&gt;=1,Q$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="R7" s="0" t="n">
-        <f aca="false">IF(AND(R$3&gt;=1,R$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(R$3&gt;=1,R$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="S7" s="0" t="n">
-        <f aca="false">IF(AND(S$3&gt;=1,S$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(S$3&gt;=1,S$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="T7" s="0" t="n">
-        <f aca="false">IF(AND(T$3&gt;=1,T$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(T$3&gt;=1,T$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>-666666.666666667</v>
       </c>
       <c r="U7" s="0" t="n">
-        <f aca="false">IF(AND(U$3&gt;=1,U$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(U$3&gt;=1,U$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="V7" s="0" t="n">
-        <f aca="false">IF(AND(V$3&gt;=1,V$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(V$3&gt;=1,V$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="W7" s="0" t="n">
-        <f aca="false">IF(AND(W$3&gt;=1,W$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(W$3&gt;=1,W$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="X7" s="0" t="n">
-        <f aca="false">IF(AND(X$3&gt;=1,X$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(X$3&gt;=1,X$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="Y7" s="0" t="n">
-        <f aca="false">IF(AND(Y$3&gt;=1,Y$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(Y$3&gt;=1,Y$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="Z7" s="0" t="n">
-        <f aca="false">IF(AND(Z$3&gt;=1,Z$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(Z$3&gt;=1,Z$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AA7" s="0" t="n">
-        <f aca="false">IF(AND(AA$3&gt;=1,AA$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AA$3&gt;=1,AA$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AB7" s="0" t="n">
-        <f aca="false">IF(AND(AB$3&gt;=1,AB$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AB$3&gt;=1,AB$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AC7" s="0" t="n">
-        <f aca="false">IF(AND(AC$3&gt;=1,AC$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AC$3&gt;=1,AC$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AD7" s="0" t="n">
-        <f aca="false">IF(AND(AD$3&gt;=1,AD$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AD$3&gt;=1,AD$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AE7" s="0" t="n">
-        <f aca="false">IF(AND(AE$3&gt;=1,AE$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AE$3&gt;=1,AE$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AF7" s="0" t="n">
-        <f aca="false">IF(AND(AF$3&gt;=1,AF$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AF$3&gt;=1,AF$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AG7" s="0" t="n">
-        <f aca="false">IF(AND(AG$3&gt;=1,AG$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AG$3&gt;=1,AG$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AH7" s="0" t="n">
-        <f aca="false">IF(AND(AH$3&gt;=1,AH$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AH$3&gt;=1,AH$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AI7" s="0" t="n">
-        <f aca="false">IF(AND(AI$3&gt;=1,AI$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AI$3&gt;=1,AI$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AJ7" s="0" t="n">
-        <f aca="false">IF(AND(AJ$3&gt;=1,AJ$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AJ$3&gt;=1,AJ$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AK7" s="0" t="n">
-        <f aca="false">IF(AND(AK$3&gt;=1,AK$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AK$3&gt;=1,AK$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AL7" s="0" t="n">
-        <f aca="false">IF(AND(AL$3&gt;=1,AL$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AL$3&gt;=1,AL$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AM7" s="0" t="n">
-        <f aca="false">IF(AND(AM$3&gt;=1,AM$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AM$3&gt;=1,AM$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AN7" s="0" t="n">
-        <f aca="false">IF(AND(AN$3&gt;=1,AN$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AN$3&gt;=1,AN$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AO7" s="0" t="n">
-        <f aca="false">IF(AND(AO$3&gt;=1,AO$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AO$3&gt;=1,AO$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AP7" s="0" t="n">
-        <f aca="false">IF(AND(AP$3&gt;=1,AP$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AP$3&gt;=1,AP$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AQ7" s="0" t="n">
-        <f aca="false">IF(AND(AQ$3&gt;=1,AQ$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AQ$3&gt;=1,AQ$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AR7" s="0" t="n">
-        <f aca="false">IF(AND(AR$3&gt;=1,AR$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AR$3&gt;=1,AR$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
       <c r="AS7" s="0" t="n">
-        <f aca="false">IF(AND(AS$3&gt;=1,AS$3&lt;=Inputs!$B$4),-Inputs!$B$3/Inputs!$B$4,0)</f>
+        <f aca="false">IF(AND(AS$3&gt;=1,AS$3&lt;=Inputs!$C$4),-Inputs!$B$3/Inputs!$C$4,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -1314,179 +1322,179 @@
         <v>27</v>
       </c>
       <c r="B8" s="0" t="n">
-        <f aca="false">IF(AND(B$3&gt;Inputs!$B$4,B$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(B$3&gt;Inputs!$C$4,B$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="C8" s="0" t="n">
-        <f aca="false">IF(AND(C$3&gt;Inputs!$B$4,C$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(C$3&gt;Inputs!$C$4,C$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="D8" s="0" t="n">
-        <f aca="false">IF(AND(D$3&gt;Inputs!$B$4,D$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(D$3&gt;Inputs!$C$4,D$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="E8" s="0" t="n">
-        <f aca="false">IF(AND(E$3&gt;Inputs!$B$4,E$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(E$3&gt;Inputs!$C$4,E$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="F8" s="0" t="n">
-        <f aca="false">IF(AND(F$3&gt;Inputs!$B$4,F$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(F$3&gt;Inputs!$C$4,F$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="G8" s="0" t="n">
-        <f aca="false">IF(AND(G$3&gt;Inputs!$B$4,G$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(G$3&gt;Inputs!$C$4,G$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="H8" s="0" t="n">
-        <f aca="false">IF(AND(H$3&gt;Inputs!$B$4,H$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(H$3&gt;Inputs!$C$4,H$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="I8" s="0" t="n">
-        <f aca="false">IF(AND(I$3&gt;Inputs!$B$4,I$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(I$3&gt;Inputs!$C$4,I$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="J8" s="0" t="n">
-        <f aca="false">IF(AND(J$3&gt;Inputs!$B$4,J$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(J$3&gt;Inputs!$C$4,J$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="K8" s="0" t="n">
-        <f aca="false">IF(AND(K$3&gt;Inputs!$B$4,K$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(K$3&gt;Inputs!$C$4,K$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="L8" s="0" t="n">
-        <f aca="false">IF(AND(L$3&gt;Inputs!$B$4,L$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(L$3&gt;Inputs!$C$4,L$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="M8" s="0" t="n">
-        <f aca="false">IF(AND(M$3&gt;Inputs!$B$4,M$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(M$3&gt;Inputs!$C$4,M$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="N8" s="0" t="n">
-        <f aca="false">IF(AND(N$3&gt;Inputs!$B$4,N$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(N$3&gt;Inputs!$C$4,N$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="O8" s="0" t="n">
-        <f aca="false">IF(AND(O$3&gt;Inputs!$B$4,O$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(O$3&gt;Inputs!$C$4,O$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="P8" s="0" t="n">
-        <f aca="false">IF(AND(P$3&gt;Inputs!$B$4,P$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(P$3&gt;Inputs!$C$4,P$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="Q8" s="0" t="n">
-        <f aca="false">IF(AND(Q$3&gt;Inputs!$B$4,Q$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(Q$3&gt;Inputs!$C$4,Q$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="R8" s="0" t="n">
-        <f aca="false">IF(AND(R$3&gt;Inputs!$B$4,R$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(R$3&gt;Inputs!$C$4,R$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="S8" s="0" t="n">
-        <f aca="false">IF(AND(S$3&gt;Inputs!$B$4,S$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(S$3&gt;Inputs!$C$4,S$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="T8" s="0" t="n">
-        <f aca="false">IF(AND(T$3&gt;Inputs!$B$4,T$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(T$3&gt;Inputs!$C$4,T$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
       <c r="U8" s="0" t="n">
-        <f aca="false">IF(AND(U$3&gt;Inputs!$B$4,U$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(U$3&gt;Inputs!$C$4,U$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="V8" s="0" t="n">
-        <f aca="false">IF(AND(V$3&gt;Inputs!$B$4,V$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(V$3&gt;Inputs!$C$4,V$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="W8" s="0" t="n">
-        <f aca="false">IF(AND(W$3&gt;Inputs!$B$4,W$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(W$3&gt;Inputs!$C$4,W$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="X8" s="0" t="n">
-        <f aca="false">IF(AND(X$3&gt;Inputs!$B$4,X$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(X$3&gt;Inputs!$C$4,X$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="Y8" s="0" t="n">
-        <f aca="false">IF(AND(Y$3&gt;Inputs!$B$4,Y$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(Y$3&gt;Inputs!$C$4,Y$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="Z8" s="0" t="n">
-        <f aca="false">IF(AND(Z$3&gt;Inputs!$B$4,Z$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(Z$3&gt;Inputs!$C$4,Z$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AA8" s="0" t="n">
-        <f aca="false">IF(AND(AA$3&gt;Inputs!$B$4,AA$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AA$3&gt;Inputs!$C$4,AA$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AB8" s="0" t="n">
-        <f aca="false">IF(AND(AB$3&gt;Inputs!$B$4,AB$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AB$3&gt;Inputs!$C$4,AB$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AC8" s="0" t="n">
-        <f aca="false">IF(AND(AC$3&gt;Inputs!$B$4,AC$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AC$3&gt;Inputs!$C$4,AC$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AD8" s="0" t="n">
-        <f aca="false">IF(AND(AD$3&gt;Inputs!$B$4,AD$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AD$3&gt;Inputs!$C$4,AD$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AE8" s="0" t="n">
-        <f aca="false">IF(AND(AE$3&gt;Inputs!$B$4,AE$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AE$3&gt;Inputs!$C$4,AE$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AF8" s="0" t="n">
-        <f aca="false">IF(AND(AF$3&gt;Inputs!$B$4,AF$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AF$3&gt;Inputs!$C$4,AF$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AG8" s="0" t="n">
-        <f aca="false">IF(AND(AG$3&gt;Inputs!$B$4,AG$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AG$3&gt;Inputs!$C$4,AG$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AH8" s="0" t="n">
-        <f aca="false">IF(AND(AH$3&gt;Inputs!$B$4,AH$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AH$3&gt;Inputs!$C$4,AH$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AI8" s="0" t="n">
-        <f aca="false">IF(AND(AI$3&gt;Inputs!$B$4,AI$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AI$3&gt;Inputs!$C$4,AI$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AJ8" s="0" t="n">
-        <f aca="false">IF(AND(AJ$3&gt;Inputs!$B$4,AJ$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AJ$3&gt;Inputs!$C$4,AJ$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AK8" s="0" t="n">
-        <f aca="false">IF(AND(AK$3&gt;Inputs!$B$4,AK$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AK$3&gt;Inputs!$C$4,AK$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AL8" s="0" t="n">
-        <f aca="false">IF(AND(AL$3&gt;Inputs!$B$4,AL$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AL$3&gt;Inputs!$C$4,AL$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AM8" s="0" t="n">
-        <f aca="false">IF(AND(AM$3&gt;Inputs!$B$4,AM$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AM$3&gt;Inputs!$C$4,AM$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AN8" s="0" t="n">
-        <f aca="false">IF(AND(AN$3&gt;Inputs!$B$4,AN$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AN$3&gt;Inputs!$C$4,AN$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AO8" s="0" t="n">
-        <f aca="false">IF(AND(AO$3&gt;Inputs!$B$4,AO$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AO$3&gt;Inputs!$C$4,AO$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AP8" s="0" t="n">
-        <f aca="false">IF(AND(AP$3&gt;Inputs!$B$4,AP$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AP$3&gt;Inputs!$C$4,AP$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AQ8" s="0" t="n">
-        <f aca="false">IF(AND(AQ$3&gt;Inputs!$B$4,AQ$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AQ$3&gt;Inputs!$C$4,AQ$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AR8" s="0" t="n">
-        <f aca="false">IF(AND(AR$3&gt;Inputs!$B$4,AR$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AR$3&gt;Inputs!$C$4,AR$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>175000</v>
       </c>
       <c r="AS8" s="0" t="n">
-        <f aca="false">IF(AND(AS$3&gt;Inputs!$B$4,AS$3&lt;=Inputs!$B$4+Inputs!$B$7),Inputs!$B$5/12,0)</f>
+        <f aca="false">IF(AND(AS$3&gt;Inputs!$C$4,AS$3&lt;=Inputs!$C$4+Inputs!$C$7),Inputs!$B$5/12,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -1495,179 +1503,179 @@
         <v>28</v>
       </c>
       <c r="B9" s="0" t="n">
-        <f aca="false">IF(B$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(B$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="C9" s="0" t="n">
-        <f aca="false">IF(C$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(C$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="D9" s="0" t="n">
-        <f aca="false">IF(D$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(D$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="E9" s="0" t="n">
-        <f aca="false">IF(E$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(E$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="F9" s="0" t="n">
-        <f aca="false">IF(F$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(F$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="G9" s="0" t="n">
-        <f aca="false">IF(G$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(G$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="H9" s="0" t="n">
-        <f aca="false">IF(H$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(H$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="I9" s="0" t="n">
-        <f aca="false">IF(I$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(I$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="J9" s="0" t="n">
-        <f aca="false">IF(J$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(J$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="K9" s="0" t="n">
-        <f aca="false">IF(K$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(K$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="L9" s="0" t="n">
-        <f aca="false">IF(L$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(L$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="M9" s="0" t="n">
-        <f aca="false">IF(M$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(M$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="N9" s="0" t="n">
-        <f aca="false">IF(N$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(N$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="O9" s="0" t="n">
-        <f aca="false">IF(O$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(O$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="P9" s="0" t="n">
-        <f aca="false">IF(P$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(P$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="Q9" s="0" t="n">
-        <f aca="false">IF(Q$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(Q$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="R9" s="0" t="n">
-        <f aca="false">IF(R$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(R$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="S9" s="0" t="n">
-        <f aca="false">IF(S$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(S$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="T9" s="0" t="n">
-        <f aca="false">IF(T$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(T$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="U9" s="0" t="n">
-        <f aca="false">IF(U$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(U$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="V9" s="0" t="n">
-        <f aca="false">IF(V$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(V$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="W9" s="0" t="n">
-        <f aca="false">IF(W$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(W$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="X9" s="0" t="n">
-        <f aca="false">IF(X$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(X$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="Y9" s="0" t="n">
-        <f aca="false">IF(Y$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(Y$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="Z9" s="0" t="n">
-        <f aca="false">IF(Z$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(Z$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AA9" s="0" t="n">
-        <f aca="false">IF(AA$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AA$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AB9" s="0" t="n">
-        <f aca="false">IF(AB$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AB$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AC9" s="0" t="n">
-        <f aca="false">IF(AC$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AC$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AD9" s="0" t="n">
-        <f aca="false">IF(AD$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AD$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AE9" s="0" t="n">
-        <f aca="false">IF(AE$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AE$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AF9" s="0" t="n">
-        <f aca="false">IF(AF$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AF$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AG9" s="0" t="n">
-        <f aca="false">IF(AG$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AG$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AH9" s="0" t="n">
-        <f aca="false">IF(AH$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AH$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AI9" s="0" t="n">
-        <f aca="false">IF(AI$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AI$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AJ9" s="0" t="n">
-        <f aca="false">IF(AJ$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AJ$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AK9" s="0" t="n">
-        <f aca="false">IF(AK$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AK$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AL9" s="0" t="n">
-        <f aca="false">IF(AL$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AL$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AM9" s="0" t="n">
-        <f aca="false">IF(AM$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AM$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AN9" s="0" t="n">
-        <f aca="false">IF(AN$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AN$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AO9" s="0" t="n">
-        <f aca="false">IF(AO$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AO$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AP9" s="0" t="n">
-        <f aca="false">IF(AP$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AP$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AQ9" s="0" t="n">
-        <f aca="false">IF(AQ$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AQ$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AR9" s="0" t="n">
-        <f aca="false">IF(AR$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AR$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="AS9" s="0" t="n">
-        <f aca="false">IF(AS$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
+        <f aca="false">IF(AS$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$5/Inputs!$B$6,0)</f>
         <v>32307692.3076923</v>
       </c>
     </row>
@@ -2223,175 +2231,175 @@
         <v>0</v>
       </c>
       <c r="C13" s="0" t="n">
-        <f aca="false">IF(C$3=Inputs!$B$4+Inputs!$B$7+1,-(B15+C11),0)</f>
+        <f aca="false">IF(C$3=Inputs!$C$4+Inputs!$C$7+1,-(B15+C11),0)</f>
         <v>0</v>
       </c>
       <c r="D13" s="0" t="n">
-        <f aca="false">IF(D$3=Inputs!$B$4+Inputs!$B$7+1,-(C15+D11),0)</f>
+        <f aca="false">IF(D$3=Inputs!$C$4+Inputs!$C$7+1,-(C15+D11),0)</f>
         <v>0</v>
       </c>
       <c r="E13" s="0" t="n">
-        <f aca="false">IF(E$3=Inputs!$B$4+Inputs!$B$7+1,-(D15+E11),0)</f>
+        <f aca="false">IF(E$3=Inputs!$C$4+Inputs!$C$7+1,-(D15+E11),0)</f>
         <v>0</v>
       </c>
       <c r="F13" s="0" t="n">
-        <f aca="false">IF(F$3=Inputs!$B$4+Inputs!$B$7+1,-(E15+F11),0)</f>
+        <f aca="false">IF(F$3=Inputs!$C$4+Inputs!$C$7+1,-(E15+F11),0)</f>
         <v>0</v>
       </c>
       <c r="G13" s="0" t="n">
-        <f aca="false">IF(G$3=Inputs!$B$4+Inputs!$B$7+1,-(F15+G11),0)</f>
+        <f aca="false">IF(G$3=Inputs!$C$4+Inputs!$C$7+1,-(F15+G11),0)</f>
         <v>0</v>
       </c>
       <c r="H13" s="0" t="n">
-        <f aca="false">IF(H$3=Inputs!$B$4+Inputs!$B$7+1,-(G15+H11),0)</f>
+        <f aca="false">IF(H$3=Inputs!$C$4+Inputs!$C$7+1,-(G15+H11),0)</f>
         <v>0</v>
       </c>
       <c r="I13" s="0" t="n">
-        <f aca="false">IF(I$3=Inputs!$B$4+Inputs!$B$7+1,-(H15+I11),0)</f>
+        <f aca="false">IF(I$3=Inputs!$C$4+Inputs!$C$7+1,-(H15+I11),0)</f>
         <v>0</v>
       </c>
       <c r="J13" s="0" t="n">
-        <f aca="false">IF(J$3=Inputs!$B$4+Inputs!$B$7+1,-(I15+J11),0)</f>
+        <f aca="false">IF(J$3=Inputs!$C$4+Inputs!$C$7+1,-(I15+J11),0)</f>
         <v>0</v>
       </c>
       <c r="K13" s="0" t="n">
-        <f aca="false">IF(K$3=Inputs!$B$4+Inputs!$B$7+1,-(J15+K11),0)</f>
+        <f aca="false">IF(K$3=Inputs!$C$4+Inputs!$C$7+1,-(J15+K11),0)</f>
         <v>0</v>
       </c>
       <c r="L13" s="0" t="n">
-        <f aca="false">IF(L$3=Inputs!$B$4+Inputs!$B$7+1,-(K15+L11),0)</f>
+        <f aca="false">IF(L$3=Inputs!$C$4+Inputs!$C$7+1,-(K15+L11),0)</f>
         <v>0</v>
       </c>
       <c r="M13" s="0" t="n">
-        <f aca="false">IF(M$3=Inputs!$B$4+Inputs!$B$7+1,-(L15+M11),0)</f>
+        <f aca="false">IF(M$3=Inputs!$C$4+Inputs!$C$7+1,-(L15+M11),0)</f>
         <v>0</v>
       </c>
       <c r="N13" s="0" t="n">
-        <f aca="false">IF(N$3=Inputs!$B$4+Inputs!$B$7+1,-(M15+N11),0)</f>
+        <f aca="false">IF(N$3=Inputs!$C$4+Inputs!$C$7+1,-(M15+N11),0)</f>
         <v>0</v>
       </c>
       <c r="O13" s="0" t="n">
-        <f aca="false">IF(O$3=Inputs!$B$4+Inputs!$B$7+1,-(N15+O11),0)</f>
+        <f aca="false">IF(O$3=Inputs!$C$4+Inputs!$C$7+1,-(N15+O11),0)</f>
         <v>0</v>
       </c>
       <c r="P13" s="0" t="n">
-        <f aca="false">IF(P$3=Inputs!$B$4+Inputs!$B$7+1,-(O15+P11),0)</f>
+        <f aca="false">IF(P$3=Inputs!$C$4+Inputs!$C$7+1,-(O15+P11),0)</f>
         <v>0</v>
       </c>
       <c r="Q13" s="0" t="n">
-        <f aca="false">IF(Q$3=Inputs!$B$4+Inputs!$B$7+1,-(P15+Q11),0)</f>
+        <f aca="false">IF(Q$3=Inputs!$C$4+Inputs!$C$7+1,-(P15+Q11),0)</f>
         <v>0</v>
       </c>
       <c r="R13" s="0" t="n">
-        <f aca="false">IF(R$3=Inputs!$B$4+Inputs!$B$7+1,-(Q15+R11),0)</f>
+        <f aca="false">IF(R$3=Inputs!$C$4+Inputs!$C$7+1,-(Q15+R11),0)</f>
         <v>0</v>
       </c>
       <c r="S13" s="0" t="n">
-        <f aca="false">IF(S$3=Inputs!$B$4+Inputs!$B$7+1,-(R15+S11),0)</f>
+        <f aca="false">IF(S$3=Inputs!$C$4+Inputs!$C$7+1,-(R15+S11),0)</f>
         <v>0</v>
       </c>
       <c r="T13" s="0" t="n">
-        <f aca="false">IF(T$3=Inputs!$B$4+Inputs!$B$7+1,-(S15+T11),0)</f>
+        <f aca="false">IF(T$3=Inputs!$C$4+Inputs!$C$7+1,-(S15+T11),0)</f>
         <v>0</v>
       </c>
       <c r="U13" s="0" t="n">
-        <f aca="false">IF(U$3=Inputs!$B$4+Inputs!$B$7+1,-(T15+U11),0)</f>
+        <f aca="false">IF(U$3=Inputs!$C$4+Inputs!$C$7+1,-(T15+U11),0)</f>
         <v>0</v>
       </c>
       <c r="V13" s="0" t="n">
-        <f aca="false">IF(V$3=Inputs!$B$4+Inputs!$B$7+1,-(U15+V11),0)</f>
+        <f aca="false">IF(V$3=Inputs!$C$4+Inputs!$C$7+1,-(U15+V11),0)</f>
         <v>0</v>
       </c>
       <c r="W13" s="0" t="n">
-        <f aca="false">IF(W$3=Inputs!$B$4+Inputs!$B$7+1,-(V15+W11),0)</f>
+        <f aca="false">IF(W$3=Inputs!$C$4+Inputs!$C$7+1,-(V15+W11),0)</f>
         <v>0</v>
       </c>
       <c r="X13" s="0" t="n">
-        <f aca="false">IF(X$3=Inputs!$B$4+Inputs!$B$7+1,-(W15+X11),0)</f>
+        <f aca="false">IF(X$3=Inputs!$C$4+Inputs!$C$7+1,-(W15+X11),0)</f>
         <v>0</v>
       </c>
       <c r="Y13" s="0" t="n">
-        <f aca="false">IF(Y$3=Inputs!$B$4+Inputs!$B$7+1,-(X15+Y11),0)</f>
+        <f aca="false">IF(Y$3=Inputs!$C$4+Inputs!$C$7+1,-(X15+Y11),0)</f>
         <v>0</v>
       </c>
       <c r="Z13" s="0" t="n">
-        <f aca="false">IF(Z$3=Inputs!$B$4+Inputs!$B$7+1,-(Y15+Z11),0)</f>
+        <f aca="false">IF(Z$3=Inputs!$C$4+Inputs!$C$7+1,-(Y15+Z11),0)</f>
         <v>0</v>
       </c>
       <c r="AA13" s="0" t="n">
-        <f aca="false">IF(AA$3=Inputs!$B$4+Inputs!$B$7+1,-(Z15+AA11),0)</f>
+        <f aca="false">IF(AA$3=Inputs!$C$4+Inputs!$C$7+1,-(Z15+AA11),0)</f>
         <v>0</v>
       </c>
       <c r="AB13" s="0" t="n">
-        <f aca="false">IF(AB$3=Inputs!$B$4+Inputs!$B$7+1,-(AA15+AB11),0)</f>
+        <f aca="false">IF(AB$3=Inputs!$C$4+Inputs!$C$7+1,-(AA15+AB11),0)</f>
         <v>0</v>
       </c>
       <c r="AC13" s="0" t="n">
-        <f aca="false">IF(AC$3=Inputs!$B$4+Inputs!$B$7+1,-(AB15+AC11),0)</f>
+        <f aca="false">IF(AC$3=Inputs!$C$4+Inputs!$C$7+1,-(AB15+AC11),0)</f>
         <v>0</v>
       </c>
       <c r="AD13" s="0" t="n">
-        <f aca="false">IF(AD$3=Inputs!$B$4+Inputs!$B$7+1,-(AC15+AD11),0)</f>
+        <f aca="false">IF(AD$3=Inputs!$C$4+Inputs!$C$7+1,-(AC15+AD11),0)</f>
         <v>0</v>
       </c>
       <c r="AE13" s="0" t="n">
-        <f aca="false">IF(AE$3=Inputs!$B$4+Inputs!$B$7+1,-(AD15+AE11),0)</f>
+        <f aca="false">IF(AE$3=Inputs!$C$4+Inputs!$C$7+1,-(AD15+AE11),0)</f>
         <v>0</v>
       </c>
       <c r="AF13" s="0" t="n">
-        <f aca="false">IF(AF$3=Inputs!$B$4+Inputs!$B$7+1,-(AE15+AF11),0)</f>
+        <f aca="false">IF(AF$3=Inputs!$C$4+Inputs!$C$7+1,-(AE15+AF11),0)</f>
         <v>0</v>
       </c>
       <c r="AG13" s="0" t="n">
-        <f aca="false">IF(AG$3=Inputs!$B$4+Inputs!$B$7+1,-(AF15+AG11),0)</f>
+        <f aca="false">IF(AG$3=Inputs!$C$4+Inputs!$C$7+1,-(AF15+AG11),0)</f>
         <v>0</v>
       </c>
       <c r="AH13" s="0" t="n">
-        <f aca="false">IF(AH$3=Inputs!$B$4+Inputs!$B$7+1,-(AG15+AH11),0)</f>
+        <f aca="false">IF(AH$3=Inputs!$C$4+Inputs!$C$7+1,-(AG15+AH11),0)</f>
         <v>0</v>
       </c>
       <c r="AI13" s="0" t="n">
-        <f aca="false">IF(AI$3=Inputs!$B$4+Inputs!$B$7+1,-(AH15+AI11),0)</f>
+        <f aca="false">IF(AI$3=Inputs!$C$4+Inputs!$C$7+1,-(AH15+AI11),0)</f>
         <v>0</v>
       </c>
       <c r="AJ13" s="0" t="n">
-        <f aca="false">IF(AJ$3=Inputs!$B$4+Inputs!$B$7+1,-(AI15+AJ11),0)</f>
+        <f aca="false">IF(AJ$3=Inputs!$C$4+Inputs!$C$7+1,-(AI15+AJ11),0)</f>
         <v>0</v>
       </c>
       <c r="AK13" s="0" t="n">
-        <f aca="false">IF(AK$3=Inputs!$B$4+Inputs!$B$7+1,-(AJ15+AK11),0)</f>
+        <f aca="false">IF(AK$3=Inputs!$C$4+Inputs!$C$7+1,-(AJ15+AK11),0)</f>
         <v>0</v>
       </c>
       <c r="AL13" s="0" t="n">
-        <f aca="false">IF(AL$3=Inputs!$B$4+Inputs!$B$7+1,-(AK15+AL11),0)</f>
+        <f aca="false">IF(AL$3=Inputs!$C$4+Inputs!$C$7+1,-(AK15+AL11),0)</f>
         <v>0</v>
       </c>
       <c r="AM13" s="0" t="n">
-        <f aca="false">IF(AM$3=Inputs!$B$4+Inputs!$B$7+1,-(AL15+AM11),0)</f>
+        <f aca="false">IF(AM$3=Inputs!$C$4+Inputs!$C$7+1,-(AL15+AM11),0)</f>
         <v>0</v>
       </c>
       <c r="AN13" s="0" t="n">
-        <f aca="false">IF(AN$3=Inputs!$B$4+Inputs!$B$7+1,-(AM15+AN11),0)</f>
+        <f aca="false">IF(AN$3=Inputs!$C$4+Inputs!$C$7+1,-(AM15+AN11),0)</f>
         <v>0</v>
       </c>
       <c r="AO13" s="0" t="n">
-        <f aca="false">IF(AO$3=Inputs!$B$4+Inputs!$B$7+1,-(AN15+AO11),0)</f>
+        <f aca="false">IF(AO$3=Inputs!$C$4+Inputs!$C$7+1,-(AN15+AO11),0)</f>
         <v>0</v>
       </c>
       <c r="AP13" s="0" t="n">
-        <f aca="false">IF(AP$3=Inputs!$B$4+Inputs!$B$7+1,-(AO15+AP11),0)</f>
+        <f aca="false">IF(AP$3=Inputs!$C$4+Inputs!$C$7+1,-(AO15+AP11),0)</f>
         <v>0</v>
       </c>
       <c r="AQ13" s="0" t="n">
-        <f aca="false">IF(AQ$3=Inputs!$B$4+Inputs!$B$7+1,-(AP15+AQ11),0)</f>
+        <f aca="false">IF(AQ$3=Inputs!$C$4+Inputs!$C$7+1,-(AP15+AQ11),0)</f>
         <v>0</v>
       </c>
       <c r="AR13" s="0" t="n">
-        <f aca="false">IF(AR$3=Inputs!$B$4+Inputs!$B$7+1,-(AQ15+AR11),0)</f>
+        <f aca="false">IF(AR$3=Inputs!$C$4+Inputs!$C$7+1,-(AQ15+AR11),0)</f>
         <v>0</v>
       </c>
       <c r="AS13" s="0" t="n">
-        <f aca="false">IF(AS$3=Inputs!$B$4+Inputs!$B$7+1,-(AR15+AS11),0)</f>
+        <f aca="false">IF(AS$3=Inputs!$C$4+Inputs!$C$7+1,-(AR15+AS11),0)</f>
         <v>-9000000</v>
       </c>
     </row>
@@ -2762,179 +2770,179 @@
         <v>35</v>
       </c>
       <c r="B17" s="0" t="n">
-        <f aca="false">B14*Inputs!$B$10-IF(B$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">B14*Inputs!$B$10-IF(B$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-1080000</v>
       </c>
       <c r="C17" s="0" t="n">
-        <f aca="false">C14*Inputs!$B$10-IF(C$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">C14*Inputs!$B$10-IF(C$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-249450</v>
       </c>
       <c r="D17" s="0" t="n">
-        <f aca="false">D14*Inputs!$B$10-IF(D$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">D14*Inputs!$B$10-IF(D$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-251550</v>
       </c>
       <c r="E17" s="0" t="n">
-        <f aca="false">E14*Inputs!$B$10-IF(E$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">E14*Inputs!$B$10-IF(E$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-253650</v>
       </c>
       <c r="F17" s="0" t="n">
-        <f aca="false">F14*Inputs!$B$10-IF(F$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">F14*Inputs!$B$10-IF(F$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-255750</v>
       </c>
       <c r="G17" s="0" t="n">
-        <f aca="false">G14*Inputs!$B$10-IF(G$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">G14*Inputs!$B$10-IF(G$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-257850</v>
       </c>
       <c r="H17" s="0" t="n">
-        <f aca="false">H14*Inputs!$B$10-IF(H$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">H14*Inputs!$B$10-IF(H$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-259950</v>
       </c>
       <c r="I17" s="0" t="n">
-        <f aca="false">I14*Inputs!$B$10-IF(I$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">I14*Inputs!$B$10-IF(I$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-262050</v>
       </c>
       <c r="J17" s="0" t="n">
-        <f aca="false">J14*Inputs!$B$10-IF(J$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">J14*Inputs!$B$10-IF(J$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-264150</v>
       </c>
       <c r="K17" s="0" t="n">
-        <f aca="false">K14*Inputs!$B$10-IF(K$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">K14*Inputs!$B$10-IF(K$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-266250</v>
       </c>
       <c r="L17" s="0" t="n">
-        <f aca="false">L14*Inputs!$B$10-IF(L$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">L14*Inputs!$B$10-IF(L$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-268350</v>
       </c>
       <c r="M17" s="0" t="n">
-        <f aca="false">M14*Inputs!$B$10-IF(M$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">M14*Inputs!$B$10-IF(M$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-270450</v>
       </c>
       <c r="N17" s="0" t="n">
-        <f aca="false">N14*Inputs!$B$10-IF(N$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">N14*Inputs!$B$10-IF(N$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-272550</v>
       </c>
       <c r="O17" s="0" t="n">
-        <f aca="false">O14*Inputs!$B$10-IF(O$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">O14*Inputs!$B$10-IF(O$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-274650</v>
       </c>
       <c r="P17" s="0" t="n">
-        <f aca="false">P14*Inputs!$B$10-IF(P$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">P14*Inputs!$B$10-IF(P$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-276750</v>
       </c>
       <c r="Q17" s="0" t="n">
-        <f aca="false">Q14*Inputs!$B$10-IF(Q$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">Q14*Inputs!$B$10-IF(Q$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-278850</v>
       </c>
       <c r="R17" s="0" t="n">
-        <f aca="false">R14*Inputs!$B$10-IF(R$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">R14*Inputs!$B$10-IF(R$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-280950</v>
       </c>
       <c r="S17" s="0" t="n">
-        <f aca="false">S14*Inputs!$B$10-IF(S$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">S14*Inputs!$B$10-IF(S$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-283050</v>
       </c>
       <c r="T17" s="0" t="n">
-        <f aca="false">T14*Inputs!$B$10-IF(T$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">T14*Inputs!$B$10-IF(T$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-285150</v>
       </c>
       <c r="U17" s="0" t="n">
-        <f aca="false">U14*Inputs!$B$10-IF(U$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">U14*Inputs!$B$10-IF(U$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="V17" s="0" t="n">
-        <f aca="false">V14*Inputs!$B$10-IF(V$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">V14*Inputs!$B$10-IF(V$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="W17" s="0" t="n">
-        <f aca="false">W14*Inputs!$B$10-IF(W$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">W14*Inputs!$B$10-IF(W$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="X17" s="0" t="n">
-        <f aca="false">X14*Inputs!$B$10-IF(X$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">X14*Inputs!$B$10-IF(X$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="Y17" s="0" t="n">
-        <f aca="false">Y14*Inputs!$B$10-IF(Y$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">Y14*Inputs!$B$10-IF(Y$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="Z17" s="0" t="n">
-        <f aca="false">Z14*Inputs!$B$10-IF(Z$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">Z14*Inputs!$B$10-IF(Z$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AA17" s="0" t="n">
-        <f aca="false">AA14*Inputs!$B$10-IF(AA$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AA14*Inputs!$B$10-IF(AA$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AB17" s="0" t="n">
-        <f aca="false">AB14*Inputs!$B$10-IF(AB$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AB14*Inputs!$B$10-IF(AB$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AC17" s="0" t="n">
-        <f aca="false">AC14*Inputs!$B$10-IF(AC$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AC14*Inputs!$B$10-IF(AC$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AD17" s="0" t="n">
-        <f aca="false">AD14*Inputs!$B$10-IF(AD$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AD14*Inputs!$B$10-IF(AD$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AE17" s="0" t="n">
-        <f aca="false">AE14*Inputs!$B$10-IF(AE$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AE14*Inputs!$B$10-IF(AE$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AF17" s="0" t="n">
-        <f aca="false">AF14*Inputs!$B$10-IF(AF$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AF14*Inputs!$B$10-IF(AF$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AG17" s="0" t="n">
-        <f aca="false">AG14*Inputs!$B$10-IF(AG$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AG14*Inputs!$B$10-IF(AG$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AH17" s="0" t="n">
-        <f aca="false">AH14*Inputs!$B$10-IF(AH$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AH14*Inputs!$B$10-IF(AH$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AI17" s="0" t="n">
-        <f aca="false">AI14*Inputs!$B$10-IF(AI$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AI14*Inputs!$B$10-IF(AI$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AJ17" s="0" t="n">
-        <f aca="false">AJ14*Inputs!$B$10-IF(AJ$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AJ14*Inputs!$B$10-IF(AJ$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AK17" s="0" t="n">
-        <f aca="false">AK14*Inputs!$B$10-IF(AK$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AK14*Inputs!$B$10-IF(AK$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AL17" s="0" t="n">
-        <f aca="false">AL14*Inputs!$B$10-IF(AL$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AL14*Inputs!$B$10-IF(AL$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AM17" s="0" t="n">
-        <f aca="false">AM14*Inputs!$B$10-IF(AM$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AM14*Inputs!$B$10-IF(AM$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AN17" s="0" t="n">
-        <f aca="false">AN14*Inputs!$B$10-IF(AN$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AN14*Inputs!$B$10-IF(AN$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AO17" s="0" t="n">
-        <f aca="false">AO14*Inputs!$B$10-IF(AO$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AO14*Inputs!$B$10-IF(AO$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AP17" s="0" t="n">
-        <f aca="false">AP14*Inputs!$B$10-IF(AP$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AP14*Inputs!$B$10-IF(AP$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AQ17" s="0" t="n">
-        <f aca="false">AQ14*Inputs!$B$10-IF(AQ$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AQ14*Inputs!$B$10-IF(AQ$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AR17" s="0" t="n">
-        <f aca="false">AR14*Inputs!$B$10-IF(AR$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AR14*Inputs!$B$10-IF(AR$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>110250</v>
       </c>
       <c r="AS17" s="0" t="n">
-        <f aca="false">AS14*Inputs!$B$10-IF(AS$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AS14*Inputs!$B$10-IF(AS$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>17392818.4615385</v>
       </c>
     </row>
@@ -2943,179 +2951,179 @@
         <v>36</v>
       </c>
       <c r="B18" s="0" t="n">
-        <f aca="false">B14*(1-Inputs!$B$10)+IF(B$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">B14*(1-Inputs!$B$10)+IF(B$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-120000</v>
       </c>
       <c r="C18" s="0" t="n">
-        <f aca="false">C14*(1-Inputs!$B$10)+IF(C$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">C14*(1-Inputs!$B$10)+IF(C$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-27716.6666666667</v>
       </c>
       <c r="D18" s="0" t="n">
-        <f aca="false">D14*(1-Inputs!$B$10)+IF(D$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">D14*(1-Inputs!$B$10)+IF(D$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-27950</v>
       </c>
       <c r="E18" s="0" t="n">
-        <f aca="false">E14*(1-Inputs!$B$10)+IF(E$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">E14*(1-Inputs!$B$10)+IF(E$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-28183.3333333333</v>
       </c>
       <c r="F18" s="0" t="n">
-        <f aca="false">F14*(1-Inputs!$B$10)+IF(F$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">F14*(1-Inputs!$B$10)+IF(F$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-28416.6666666667</v>
       </c>
       <c r="G18" s="0" t="n">
-        <f aca="false">G14*(1-Inputs!$B$10)+IF(G$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">G14*(1-Inputs!$B$10)+IF(G$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-28650</v>
       </c>
       <c r="H18" s="0" t="n">
-        <f aca="false">H14*(1-Inputs!$B$10)+IF(H$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">H14*(1-Inputs!$B$10)+IF(H$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-28883.3333333333</v>
       </c>
       <c r="I18" s="0" t="n">
-        <f aca="false">I14*(1-Inputs!$B$10)+IF(I$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">I14*(1-Inputs!$B$10)+IF(I$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-29116.6666666667</v>
       </c>
       <c r="J18" s="0" t="n">
-        <f aca="false">J14*(1-Inputs!$B$10)+IF(J$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">J14*(1-Inputs!$B$10)+IF(J$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-29350</v>
       </c>
       <c r="K18" s="0" t="n">
-        <f aca="false">K14*(1-Inputs!$B$10)+IF(K$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">K14*(1-Inputs!$B$10)+IF(K$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-29583.3333333333</v>
       </c>
       <c r="L18" s="0" t="n">
-        <f aca="false">L14*(1-Inputs!$B$10)+IF(L$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">L14*(1-Inputs!$B$10)+IF(L$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-29816.6666666667</v>
       </c>
       <c r="M18" s="0" t="n">
-        <f aca="false">M14*(1-Inputs!$B$10)+IF(M$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">M14*(1-Inputs!$B$10)+IF(M$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-30050</v>
       </c>
       <c r="N18" s="0" t="n">
-        <f aca="false">N14*(1-Inputs!$B$10)+IF(N$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">N14*(1-Inputs!$B$10)+IF(N$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-30283.3333333333</v>
       </c>
       <c r="O18" s="0" t="n">
-        <f aca="false">O14*(1-Inputs!$B$10)+IF(O$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">O14*(1-Inputs!$B$10)+IF(O$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-30516.6666666667</v>
       </c>
       <c r="P18" s="0" t="n">
-        <f aca="false">P14*(1-Inputs!$B$10)+IF(P$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">P14*(1-Inputs!$B$10)+IF(P$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-30750</v>
       </c>
       <c r="Q18" s="0" t="n">
-        <f aca="false">Q14*(1-Inputs!$B$10)+IF(Q$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">Q14*(1-Inputs!$B$10)+IF(Q$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-30983.3333333333</v>
       </c>
       <c r="R18" s="0" t="n">
-        <f aca="false">R14*(1-Inputs!$B$10)+IF(R$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">R14*(1-Inputs!$B$10)+IF(R$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-31216.6666666667</v>
       </c>
       <c r="S18" s="0" t="n">
-        <f aca="false">S14*(1-Inputs!$B$10)+IF(S$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">S14*(1-Inputs!$B$10)+IF(S$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-31450</v>
       </c>
       <c r="T18" s="0" t="n">
-        <f aca="false">T14*(1-Inputs!$B$10)+IF(T$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">T14*(1-Inputs!$B$10)+IF(T$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>-31683.3333333333</v>
       </c>
       <c r="U18" s="0" t="n">
-        <f aca="false">U14*(1-Inputs!$B$10)+IF(U$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">U14*(1-Inputs!$B$10)+IF(U$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="V18" s="0" t="n">
-        <f aca="false">V14*(1-Inputs!$B$10)+IF(V$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">V14*(1-Inputs!$B$10)+IF(V$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="W18" s="0" t="n">
-        <f aca="false">W14*(1-Inputs!$B$10)+IF(W$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">W14*(1-Inputs!$B$10)+IF(W$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="X18" s="0" t="n">
-        <f aca="false">X14*(1-Inputs!$B$10)+IF(X$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">X14*(1-Inputs!$B$10)+IF(X$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="Y18" s="0" t="n">
-        <f aca="false">Y14*(1-Inputs!$B$10)+IF(Y$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">Y14*(1-Inputs!$B$10)+IF(Y$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="Z18" s="0" t="n">
-        <f aca="false">Z14*(1-Inputs!$B$10)+IF(Z$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">Z14*(1-Inputs!$B$10)+IF(Z$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AA18" s="0" t="n">
-        <f aca="false">AA14*(1-Inputs!$B$10)+IF(AA$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AA14*(1-Inputs!$B$10)+IF(AA$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AB18" s="0" t="n">
-        <f aca="false">AB14*(1-Inputs!$B$10)+IF(AB$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AB14*(1-Inputs!$B$10)+IF(AB$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AC18" s="0" t="n">
-        <f aca="false">AC14*(1-Inputs!$B$10)+IF(AC$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AC14*(1-Inputs!$B$10)+IF(AC$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AD18" s="0" t="n">
-        <f aca="false">AD14*(1-Inputs!$B$10)+IF(AD$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AD14*(1-Inputs!$B$10)+IF(AD$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AE18" s="0" t="n">
-        <f aca="false">AE14*(1-Inputs!$B$10)+IF(AE$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AE14*(1-Inputs!$B$10)+IF(AE$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AF18" s="0" t="n">
-        <f aca="false">AF14*(1-Inputs!$B$10)+IF(AF$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AF14*(1-Inputs!$B$10)+IF(AF$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AG18" s="0" t="n">
-        <f aca="false">AG14*(1-Inputs!$B$10)+IF(AG$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AG14*(1-Inputs!$B$10)+IF(AG$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AH18" s="0" t="n">
-        <f aca="false">AH14*(1-Inputs!$B$10)+IF(AH$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AH14*(1-Inputs!$B$10)+IF(AH$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AI18" s="0" t="n">
-        <f aca="false">AI14*(1-Inputs!$B$10)+IF(AI$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AI14*(1-Inputs!$B$10)+IF(AI$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AJ18" s="0" t="n">
-        <f aca="false">AJ14*(1-Inputs!$B$10)+IF(AJ$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AJ14*(1-Inputs!$B$10)+IF(AJ$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AK18" s="0" t="n">
-        <f aca="false">AK14*(1-Inputs!$B$10)+IF(AK$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AK14*(1-Inputs!$B$10)+IF(AK$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AL18" s="0" t="n">
-        <f aca="false">AL14*(1-Inputs!$B$10)+IF(AL$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AL14*(1-Inputs!$B$10)+IF(AL$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AM18" s="0" t="n">
-        <f aca="false">AM14*(1-Inputs!$B$10)+IF(AM$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AM14*(1-Inputs!$B$10)+IF(AM$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AN18" s="0" t="n">
-        <f aca="false">AN14*(1-Inputs!$B$10)+IF(AN$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AN14*(1-Inputs!$B$10)+IF(AN$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AO18" s="0" t="n">
-        <f aca="false">AO14*(1-Inputs!$B$10)+IF(AO$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AO14*(1-Inputs!$B$10)+IF(AO$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AP18" s="0" t="n">
-        <f aca="false">AP14*(1-Inputs!$B$10)+IF(AP$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AP14*(1-Inputs!$B$10)+IF(AP$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AQ18" s="0" t="n">
-        <f aca="false">AQ14*(1-Inputs!$B$10)+IF(AQ$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AQ14*(1-Inputs!$B$10)+IF(AQ$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AR18" s="0" t="n">
-        <f aca="false">AR14*(1-Inputs!$B$10)+IF(AR$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AR14*(1-Inputs!$B$10)+IF(AR$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>12250</v>
       </c>
       <c r="AS18" s="0" t="n">
-        <f aca="false">AS14*(1-Inputs!$B$10)+IF(AS$3=Inputs!$B$4+Inputs!$B$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
+        <f aca="false">AS14*(1-Inputs!$B$10)+IF(AS$3=Inputs!$C$4+Inputs!$C$7+1,Inputs!$B$12*MAX(0,SUM($B$14:$AS$14))*Inputs!$B$10,0)</f>
         <v>5862373.84615385</v>
       </c>
     </row>

</xml_diff>